<commit_message>
RTP baseline and error fix for TOU8
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
@@ -8,9 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\sweep results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AC3565F-11BF-4838-AF9A-FB0F5E3F0EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9868276-1B3B-4482-8D6A-72B457499567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-6375" yWindow="-21600" windowWidth="14175" windowHeight="20985" firstSheet="1" activeTab="2" xr2:uid="{526C491F-7D81-4CF8-8DF5-6D840C914C1B}"/>
+    <workbookView xWindow="14503" yWindow="0" windowWidth="18497" windowHeight="17880" activeTab="2" xr2:uid="{526C491F-7D81-4CF8-8DF5-6D840C914C1B}"/>
+    <workbookView xWindow="-86" yWindow="0" windowWidth="14760" windowHeight="17880" activeTab="1" xr2:uid="{811D88E6-5E04-4AC4-9B26-930D2EA2E3F2}"/>
   </bookViews>
   <sheets>
     <sheet name="Summer Cost Summary" sheetId="4" r:id="rId1"/>
@@ -92,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="27">
   <si>
     <t>Annual AF</t>
   </si>
@@ -292,8 +293,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}" name="Table1" displayName="Table1" ref="A1:Q33" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:Q33" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}" name="Table1" displayName="Table1" ref="A1:Q39" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:Q39" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}">
     <filterColumn colId="0">
       <filters>
         <filter val="Winter"/>
@@ -301,12 +302,12 @@
     </filterColumn>
     <filterColumn colId="1">
       <filters>
-        <filter val="3"/>
+        <filter val="0"/>
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q24">
-    <sortCondition ref="D1:D24"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q39">
+    <sortCondition ref="D1:D39"/>
   </sortState>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{FADC07E8-CEDF-4B75-BBE4-A01ACB71EDD0}" name="Season"/>
@@ -619,24 +620,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B1DDFCB-CD48-4284-8222-18B5894FE623}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="9.23046875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.4609375" customWidth="1"/>
-    <col min="4" max="4" width="9.84375" customWidth="1"/>
-    <col min="5" max="5" width="9.4609375" customWidth="1"/>
-    <col min="6" max="6" width="10.3828125" customWidth="1"/>
+    <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.453125" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" customWidth="1"/>
+    <col min="5" max="5" width="9.453125" customWidth="1"/>
+    <col min="6" max="6" width="10.36328125" customWidth="1"/>
     <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D2">
         <v>0</v>
       </c>
@@ -647,7 +648,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>0</v>
       </c>
@@ -655,7 +656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -669,7 +670,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B5" s="3">
         <f>C5/$G$10</f>
         <v>1798.4286079070769</v>
@@ -680,7 +681,7 @@
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B6" s="3">
         <f>C6/$G$10</f>
         <v>2397.9615120043568</v>
@@ -690,22 +691,22 @@
       </c>
       <c r="D6" s="1"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D7" s="1"/>
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D8" s="1"/>
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="D9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B10">
         <v>8000</v>
       </c>
@@ -721,7 +722,7 @@
         <v>23.514972912500003</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B11">
         <v>9000</v>
       </c>
@@ -733,7 +734,7 @@
       </c>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B12" s="3">
         <f>C12/$G$10</f>
         <v>9591.8460480174272</v>
@@ -744,7 +745,7 @@
       <c r="D12" s="1"/>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B13">
         <v>10000</v>
       </c>
@@ -757,7 +758,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B14">
         <v>11000</v>
       </c>
@@ -770,7 +771,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B15">
         <v>12000</v>
       </c>
@@ -783,7 +784,7 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="B16">
         <v>13000</v>
       </c>
@@ -796,7 +797,7 @@
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B17">
         <v>14000</v>
       </c>
@@ -809,7 +810,7 @@
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B18">
         <v>15000</v>
       </c>
@@ -822,7 +823,7 @@
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="B19">
         <v>16000</v>
       </c>
@@ -835,7 +836,7 @@
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>3</v>
       </c>
@@ -852,7 +853,7 @@
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="C21">
         <f>C20*4/7</f>
         <v>225552</v>
@@ -870,23 +871,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E02D5E1-F801-4839-8C05-CA5C31CB2DFA}">
   <dimension ref="B1:H22"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="9.23046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.4609375" customWidth="1"/>
-    <col min="5" max="5" width="9.84375" customWidth="1"/>
-    <col min="6" max="6" width="9.4609375" customWidth="1"/>
-    <col min="7" max="7" width="10.3828125" customWidth="1"/>
+    <col min="3" max="3" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.453125" customWidth="1"/>
+    <col min="5" max="5" width="9.81640625" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" customWidth="1"/>
+    <col min="7" max="7" width="10.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="1" spans="2:8" x14ac:dyDescent="0.35">
       <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
     </row>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
       <c r="E2">
         <v>0</v>
       </c>
@@ -897,7 +898,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C3" t="s">
         <v>0</v>
       </c>
@@ -905,7 +906,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>4</v>
       </c>
@@ -921,7 +922,7 @@
         <v>16720.240035535448</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C5">
         <v>1798</v>
       </c>
@@ -934,7 +935,7 @@
         <v>22368.52857086459</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C6">
         <v>2398</v>
       </c>
@@ -947,7 +948,7 @@
         <v>28772.571914996501</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C7">
         <v>3000</v>
       </c>
@@ -956,7 +957,7 @@
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C8">
         <v>4000</v>
       </c>
@@ -969,7 +970,7 @@
       </c>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C9">
         <v>5000</v>
       </c>
@@ -982,7 +983,7 @@
       </c>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C10">
         <v>6000</v>
       </c>
@@ -998,7 +999,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C11">
         <v>7000</v>
       </c>
@@ -1011,12 +1012,15 @@
       </c>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C12">
         <v>8000</v>
       </c>
       <c r="D12" s="3">
         <v>188119.780821792</v>
+      </c>
+      <c r="E12">
+        <v>75507</v>
       </c>
       <c r="F12" s="3">
         <v>80116.314065181752</v>
@@ -1027,7 +1031,7 @@
         <v>23.514972602724001</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C13">
         <v>9000</v>
       </c>
@@ -1042,7 +1046,7 @@
       </c>
       <c r="G13" s="1"/>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C14" s="3">
         <f>D14/H12</f>
         <v>9591.8461743762273</v>
@@ -1053,35 +1057,47 @@
       <c r="E14" s="1"/>
       <c r="G14" s="1"/>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C15">
         <v>10000</v>
       </c>
+      <c r="E15">
+        <v>93848</v>
+      </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
       <c r="C16">
         <v>11000</v>
       </c>
+      <c r="E16" s="3">
+        <v>102961.15922754805</v>
+      </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C17">
         <v>12000</v>
       </c>
+      <c r="E17">
+        <v>112554.99851567688</v>
+      </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C18">
         <v>13000</v>
       </c>
+      <c r="E18" s="3">
+        <v>121344.56621300505</v>
+      </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C19">
         <v>14000</v>
       </c>
@@ -1094,21 +1110,27 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C20">
         <v>15000</v>
       </c>
+      <c r="E20" s="3">
+        <v>140645.20979357499</v>
+      </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C21">
         <v>16000</v>
       </c>
+      <c r="E21" s="3">
+        <v>149838.83143944858</v>
+      </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.4">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>3</v>
       </c>
@@ -1135,28 +1157,28 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44889D92-5C1B-43B6-BE00-3D23C35CC93C}">
-  <dimension ref="A1:Q33"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:Q39"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.69140625" customWidth="1"/>
-    <col min="2" max="3" width="11.84375" customWidth="1"/>
-    <col min="4" max="4" width="22.23046875" customWidth="1"/>
-    <col min="5" max="5" width="28.84375" customWidth="1"/>
-    <col min="6" max="6" width="26.921875" customWidth="1"/>
+    <col min="1" max="1" width="8.7265625" customWidth="1"/>
+    <col min="2" max="3" width="11.81640625" customWidth="1"/>
+    <col min="4" max="4" width="22.26953125" customWidth="1"/>
+    <col min="5" max="5" width="28.81640625" customWidth="1"/>
+    <col min="6" max="6" width="26.90625" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="20.07421875" customWidth="1"/>
-    <col min="9" max="9" width="21.53515625" customWidth="1"/>
-    <col min="10" max="10" width="18.4609375" customWidth="1"/>
-    <col min="11" max="11" width="18.84375" customWidth="1"/>
+    <col min="8" max="8" width="20.08984375" customWidth="1"/>
+    <col min="9" max="9" width="21.54296875" customWidth="1"/>
+    <col min="10" max="10" width="18.453125" customWidth="1"/>
+    <col min="11" max="11" width="18.81640625" customWidth="1"/>
     <col min="12" max="12" width="22" customWidth="1"/>
-    <col min="13" max="13" width="22.53515625" customWidth="1"/>
-    <col min="14" max="14" width="25.3828125" customWidth="1"/>
-    <col min="15" max="15" width="19.15234375" customWidth="1"/>
-    <col min="16" max="16" width="28.61328125" customWidth="1"/>
-    <col min="17" max="17" width="16.23046875" style="3" customWidth="1"/>
+    <col min="13" max="13" width="22.54296875" customWidth="1"/>
+    <col min="14" max="14" width="25.36328125" customWidth="1"/>
+    <col min="15" max="15" width="19.1796875" customWidth="1"/>
+    <col min="16" max="16" width="28.6328125" customWidth="1"/>
+    <col min="17" max="17" width="16.26953125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
@@ -1209,7 +1231,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1217,7 +1239,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="3">
-        <f t="shared" ref="C2:C24" si="0">N2+M2+L2+K2+J2</f>
+        <f>N2+M2+L2+K2+J2</f>
         <v>158104.1957609462</v>
       </c>
       <c r="D2">
@@ -1263,7 +1285,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1271,7 +1293,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="3">
-        <f t="shared" si="0"/>
+        <f>N3+M3+L3+K3+J3</f>
         <v>171053.54809522501</v>
       </c>
       <c r="D3">
@@ -1317,7 +1339,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1325,7 +1347,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="3">
-        <f t="shared" si="0"/>
+        <f>N4+M4+L4+K4+J4</f>
         <v>80541.55863</v>
       </c>
       <c r="D4">
@@ -1371,7 +1393,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1379,7 +1401,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="3">
-        <f t="shared" si="0"/>
+        <f>N5+M5+L5+K5+J5</f>
         <v>90145.456985227414</v>
       </c>
       <c r="D5">
@@ -1425,7 +1447,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1433,7 +1455,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="3">
-        <f t="shared" si="0"/>
+        <f>N6+M6+L6+K6+J6</f>
         <v>99135.784106883366</v>
       </c>
       <c r="D6">
@@ -1479,7 +1501,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1487,7 +1509,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="3">
-        <f t="shared" si="0"/>
+        <f>N7+M7+L7+K7+J7</f>
         <v>28772.571914996501</v>
       </c>
       <c r="D7">
@@ -1530,7 +1552,7 @@
         <v>2.6406704469603199</v>
       </c>
     </row>
-    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1538,7 +1560,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="3">
-        <f t="shared" si="0"/>
+        <f>N8+M8+L8+K8+J8</f>
         <v>22368.52857086459</v>
       </c>
       <c r="D8">
@@ -1581,7 +1603,7 @@
         <v>3.36954571208561</v>
       </c>
     </row>
-    <row r="9" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1589,7 +1611,7 @@
         <v>5</v>
       </c>
       <c r="C9" s="3">
-        <f t="shared" si="0"/>
+        <f>N9+M9+L9+K9+J9</f>
         <v>16720.240035535448</v>
       </c>
       <c r="D9">
@@ -1632,7 +1654,7 @@
         <v>4.8864727960722396</v>
       </c>
     </row>
-    <row r="10" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1640,7 +1662,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="3">
-        <f t="shared" si="0"/>
+        <f>N10+M10+L10+K10+J10</f>
         <v>108042.46335199999</v>
       </c>
       <c r="D10">
@@ -1686,7 +1708,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1694,7 +1716,7 @@
         <v>3</v>
       </c>
       <c r="C11" s="3">
-        <f t="shared" si="0"/>
+        <f>N11+M11+L11+K11+J11</f>
         <v>41752.231305558547</v>
       </c>
       <c r="D11">
@@ -1737,7 +1759,7 @@
         <v>1.7211299327173799</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -1745,7 +1767,7 @@
         <v>3</v>
       </c>
       <c r="C12" s="3">
-        <f t="shared" si="0"/>
+        <f>N12+M12+L12+K12+J12</f>
         <v>51495.778789739757</v>
       </c>
       <c r="D12">
@@ -1788,7 +1810,7 @@
         <v>1.45968753918303</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1796,7 +1818,7 @@
         <v>3</v>
       </c>
       <c r="C13" s="3">
-        <f t="shared" si="0"/>
+        <f>N13+M13+L13+K13+J13</f>
         <v>60724.979693855727</v>
       </c>
       <c r="D13">
@@ -1839,7 +1861,7 @@
         <v>1.2818199310829099</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -1847,7 +1869,7 @@
         <v>3</v>
       </c>
       <c r="C14" s="3">
-        <f t="shared" si="0"/>
+        <f>N14+M14+L14+K14+J14</f>
         <v>70388.430895292957</v>
       </c>
       <c r="D14">
@@ -1890,7 +1912,7 @@
         <v>1.15734642471583</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1898,7 +1920,7 @@
         <v>3</v>
       </c>
       <c r="C15" s="3">
-        <f t="shared" si="0"/>
+        <f>N15+M15+L15+K15+J15</f>
         <v>80116.314065181752</v>
       </c>
       <c r="D15">
@@ -1941,7 +1963,7 @@
         <v>1.06438923423513</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -1949,7 +1971,7 @@
         <v>3</v>
       </c>
       <c r="C16" s="3">
-        <f t="shared" si="0"/>
+        <f>N16+M16+L16+K16+J16</f>
         <v>90891.797768890829</v>
       </c>
       <c r="D16">
@@ -1992,7 +2014,7 @@
         <v>0.99711288227329198</v>
       </c>
     </row>
-    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -2000,7 +2022,7 @@
         <v>0</v>
       </c>
       <c r="C17" s="3">
-        <f t="shared" si="0"/>
+        <f>N17+M17+L17+K17+J17</f>
         <v>117856.65704778227</v>
       </c>
       <c r="D17">
@@ -2046,7 +2068,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -2054,7 +2076,7 @@
         <v>0</v>
       </c>
       <c r="C18" s="3">
-        <f t="shared" si="0"/>
+        <f>N18+M18+L18+K18+J18</f>
         <v>126980.73146875472</v>
       </c>
       <c r="D18">
@@ -2100,7 +2122,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -2108,7 +2130,7 @@
         <v>0</v>
       </c>
       <c r="C19" s="3">
-        <f t="shared" si="0"/>
+        <f>N19+M19+L19+K19+J19</f>
         <v>135947.17095224367</v>
       </c>
       <c r="D19">
@@ -2154,7 +2176,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2162,7 +2184,7 @@
         <v>0</v>
       </c>
       <c r="C20" s="3">
-        <f t="shared" si="0"/>
+        <f>N20+M20+L20+K20+J20</f>
         <v>75506.612155252791</v>
       </c>
       <c r="D20">
@@ -2208,7 +2230,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -2216,7 +2238,7 @@
         <v>0</v>
       </c>
       <c r="C21" s="3">
-        <f t="shared" si="0"/>
+        <f>N21+M21+L21+K21+J21</f>
         <v>85155.50909649636</v>
       </c>
       <c r="D21">
@@ -2262,7 +2284,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -2270,7 +2292,7 @@
         <v>0</v>
       </c>
       <c r="C22" s="3">
-        <f t="shared" si="0"/>
+        <f>N22+M22+L22+K22+J22</f>
         <v>146231.12922675692</v>
       </c>
       <c r="D22">
@@ -2316,7 +2338,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -2324,7 +2346,7 @@
         <v>0</v>
       </c>
       <c r="C23" s="3">
-        <f t="shared" si="0"/>
+        <f>N23+M23+L23+K23+J23</f>
         <v>159412.81974307698</v>
       </c>
       <c r="D23">
@@ -2370,7 +2392,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>19</v>
       </c>
@@ -2378,53 +2400,53 @@
         <v>0</v>
       </c>
       <c r="C24" s="3">
-        <f t="shared" si="0"/>
-        <v>130424.39365381806</v>
+        <f>N24+M24+L24+K24+J24</f>
+        <v>93848.445066986911</v>
       </c>
       <c r="D24">
-        <v>14000</v>
+        <v>10000</v>
       </c>
       <c r="E24">
         <v>10</v>
       </c>
       <c r="F24">
-        <v>329240.017626649</v>
+        <v>235174.795346464</v>
       </c>
       <c r="G24">
-        <v>250530.167023805</v>
+        <v>213972.635897431</v>
       </c>
       <c r="H24">
-        <v>20848.0798472356</v>
+        <v>14616.4032867845</v>
       </c>
       <c r="I24">
-        <v>8176.7344208997802</v>
+        <v>6351.5554479330704</v>
       </c>
       <c r="J24">
-        <v>59388.995445909903</v>
+        <v>42435.799224394301</v>
       </c>
       <c r="K24">
-        <v>18034.7176814257</v>
+        <v>12921.0484166359</v>
       </c>
       <c r="L24">
-        <v>22529.657101452402</v>
+        <v>16095.846994802199</v>
       </c>
       <c r="M24">
-        <v>29024.8142681354</v>
+        <v>20967.958734717598</v>
       </c>
       <c r="N24">
-        <v>1446.20915689464</v>
+        <v>1427.7916964369099</v>
       </c>
       <c r="O24">
-        <v>0.25149700598802299</v>
+        <v>0.125748502994011</v>
       </c>
       <c r="P24">
-        <v>0.76093473943346901</v>
+        <v>0.90984510301030797</v>
       </c>
       <c r="Q24" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -2432,7 +2454,7 @@
         <v>0</v>
       </c>
       <c r="C25" s="3">
-        <f t="shared" ref="C25:C33" si="1">N25+M25+L25+K25+J25</f>
+        <f>N25+M25+L25+K25+J25</f>
         <v>81475.122661244794</v>
       </c>
       <c r="D25">
@@ -2478,7 +2500,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -2486,7 +2508,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="3">
-        <f t="shared" si="1"/>
+        <f>N26+M26+L26+K26+J26</f>
         <v>120337.96252123939</v>
       </c>
       <c r="D26">
@@ -2532,7 +2554,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -2540,7 +2562,7 @@
         <v>0</v>
       </c>
       <c r="C27" s="3">
-        <f t="shared" si="1"/>
+        <f>N27+M27+L27+K27+J27</f>
         <v>120337.96252123939</v>
       </c>
       <c r="D27">
@@ -2586,7 +2608,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -2594,7 +2616,7 @@
         <v>0</v>
       </c>
       <c r="C28" s="3">
-        <f t="shared" si="1"/>
+        <f>N28+M28+L28+K28+J28</f>
         <v>120337.96252123939</v>
       </c>
       <c r="D28">
@@ -2640,7 +2662,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>21</v>
       </c>
@@ -2648,7 +2670,7 @@
         <v>0</v>
       </c>
       <c r="C29" s="3">
-        <f t="shared" si="1"/>
+        <f>N29+M29+L29+K29+J29</f>
         <v>121509.10762980059</v>
       </c>
       <c r="D29">
@@ -2694,7 +2716,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -2702,7 +2724,7 @@
         <v>0</v>
       </c>
       <c r="C30" s="3">
-        <f t="shared" si="1"/>
+        <f>N30+M30+L30+K30+J30</f>
         <v>160240.68755374721</v>
       </c>
       <c r="D30">
@@ -2748,7 +2770,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -2756,7 +2778,7 @@
         <v>0</v>
       </c>
       <c r="C31" s="3">
-        <f t="shared" si="1"/>
+        <f>N31+M31+L31+K31+J31</f>
         <v>160240.68755374721</v>
       </c>
       <c r="D31">
@@ -2802,7 +2824,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>21</v>
       </c>
@@ -2810,7 +2832,7 @@
         <v>0</v>
       </c>
       <c r="C32" s="3">
-        <f t="shared" si="1"/>
+        <f>N32+M32+L32+K32+J32</f>
         <v>160240.68755374721</v>
       </c>
       <c r="D32">
@@ -2856,7 +2878,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>21</v>
       </c>
@@ -2864,7 +2886,7 @@
         <v>0</v>
       </c>
       <c r="C33" s="3">
-        <f t="shared" si="1"/>
+        <f>N33+M33+L33+K33+J33</f>
         <v>161854.2162878394</v>
       </c>
       <c r="D33">
@@ -2908,6 +2930,328 @@
       </c>
       <c r="Q33" s="3" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>19</v>
+      </c>
+      <c r="B34">
+        <v>0</v>
+      </c>
+      <c r="C34" s="3">
+        <f>N34+M34+L34+K34+J34</f>
+        <v>102961.15922754805</v>
+      </c>
+      <c r="D34">
+        <v>11000</v>
+      </c>
+      <c r="E34">
+        <v>10</v>
+      </c>
+      <c r="F34">
+        <v>258664.698630136</v>
+      </c>
+      <c r="G34">
+        <v>223080.13596780499</v>
+      </c>
+      <c r="H34">
+        <v>16558.382878249799</v>
+      </c>
+      <c r="I34">
+        <v>6639.1612289695604</v>
+      </c>
+      <c r="J34">
+        <v>46607.913757927803</v>
+      </c>
+      <c r="K34">
+        <v>14032.947813471899</v>
+      </c>
+      <c r="L34">
+        <v>17689.7477623042</v>
+      </c>
+      <c r="M34">
+        <v>23197.544107219401</v>
+      </c>
+      <c r="N34">
+        <v>1433.00578662475</v>
+      </c>
+      <c r="O34">
+        <v>0.16167664670658599</v>
+      </c>
+      <c r="P34">
+        <v>0.86242976776195501</v>
+      </c>
+      <c r="Q34" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>19</v>
+      </c>
+      <c r="B35">
+        <v>0</v>
+      </c>
+      <c r="C35" s="3">
+        <f>N35+M35+L35+K35+J35</f>
+        <v>112554.99851567688</v>
+      </c>
+      <c r="D35">
+        <v>12000</v>
+      </c>
+      <c r="E35">
+        <v>10</v>
+      </c>
+      <c r="F35">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="H35">
+        <v>18242.5461916684</v>
+      </c>
+      <c r="I35">
+        <f>4852+2606</f>
+        <v>7458</v>
+      </c>
+      <c r="J35">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="K35">
+        <v>15303.798385783</v>
+      </c>
+      <c r="L35">
+        <v>19297.5304894482</v>
+      </c>
+      <c r="M35">
+        <v>25700.648204926601</v>
+      </c>
+      <c r="N35">
+        <v>1409.83742959549</v>
+      </c>
+      <c r="O35">
+        <v>0</v>
+      </c>
+      <c r="P35">
+        <v>0.82464177024617602</v>
+      </c>
+      <c r="Q35" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>19</v>
+      </c>
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36" s="3">
+        <f>N36+M36+L36+K36+J36</f>
+        <v>121344.56621300505</v>
+      </c>
+      <c r="D36">
+        <v>13000</v>
+      </c>
+      <c r="E36">
+        <v>10</v>
+      </c>
+      <c r="F36">
+        <v>305700.960485827</v>
+      </c>
+      <c r="G36">
+        <v>241450.33958299199</v>
+      </c>
+      <c r="H36">
+        <v>18893.080794400601</v>
+      </c>
+      <c r="I36">
+        <v>7655.3649078774997</v>
+      </c>
+      <c r="J36">
+        <v>55282.309265125899</v>
+      </c>
+      <c r="K36">
+        <v>17119.793141132199</v>
+      </c>
+      <c r="L36">
+        <v>20947.808947574202</v>
+      </c>
+      <c r="M36">
+        <v>26548.445702278099</v>
+      </c>
+      <c r="N36">
+        <v>1446.20915689464</v>
+      </c>
+      <c r="O36">
+        <v>0.25149700598802299</v>
+      </c>
+      <c r="P36">
+        <v>0.78982525667983905</v>
+      </c>
+      <c r="Q36" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>19</v>
+      </c>
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37" s="3">
+        <f>N37+M37+L37+K37+J37</f>
+        <v>130424.39365381806</v>
+      </c>
+      <c r="D37">
+        <v>14000</v>
+      </c>
+      <c r="E37">
+        <v>10</v>
+      </c>
+      <c r="F37">
+        <v>329240.017626649</v>
+      </c>
+      <c r="G37">
+        <v>250530.167023805</v>
+      </c>
+      <c r="H37">
+        <v>20848.0798472356</v>
+      </c>
+      <c r="I37">
+        <v>8176.7344208997802</v>
+      </c>
+      <c r="J37">
+        <v>59388.995445909903</v>
+      </c>
+      <c r="K37">
+        <v>18034.7176814257</v>
+      </c>
+      <c r="L37">
+        <v>22529.657101452402</v>
+      </c>
+      <c r="M37">
+        <v>29024.8142681354</v>
+      </c>
+      <c r="N37">
+        <v>1446.20915689464</v>
+      </c>
+      <c r="O37">
+        <v>0.25149700598802299</v>
+      </c>
+      <c r="P37">
+        <v>0.76093473943346901</v>
+      </c>
+      <c r="Q37" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>19</v>
+      </c>
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38" s="3">
+        <f>N38+M38+L38+K38+J38</f>
+        <v>140645.20979357499</v>
+      </c>
+      <c r="D38">
+        <v>15000</v>
+      </c>
+      <c r="E38">
+        <v>10</v>
+      </c>
+      <c r="F38">
+        <v>352724.58906748501</v>
+      </c>
+      <c r="G38">
+        <v>260787.354890861</v>
+      </c>
+      <c r="H38">
+        <v>22262.8898201671</v>
+      </c>
+      <c r="I38">
+        <v>9101.7415334445996</v>
+      </c>
+      <c r="J38">
+        <v>63827.433131782796</v>
+      </c>
+      <c r="K38">
+        <v>19864.653242648001</v>
+      </c>
+      <c r="L38">
+        <v>24178.654635937</v>
+      </c>
+      <c r="M38">
+        <v>31364.631353611701</v>
+      </c>
+      <c r="N38">
+        <v>1409.83742959549</v>
+      </c>
+      <c r="O38">
+        <v>0</v>
+      </c>
+      <c r="P38">
+        <v>0.73935121897885603</v>
+      </c>
+      <c r="Q38" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>19</v>
+      </c>
+      <c r="B39">
+        <v>0</v>
+      </c>
+      <c r="C39" s="3">
+        <f>N39+M39+L39+K39+J39</f>
+        <v>149838.83143944858</v>
+      </c>
+      <c r="D39">
+        <v>16000</v>
+      </c>
+      <c r="E39">
+        <v>10</v>
+      </c>
+      <c r="F39">
+        <v>376239.56164383498</v>
+      </c>
+      <c r="G39">
+        <v>269980.97653673397</v>
+      </c>
+      <c r="H39">
+        <v>24490.5164898455</v>
+      </c>
+      <c r="I39">
+        <v>10012.4603452017</v>
+      </c>
+      <c r="J39">
+        <v>67790.912007917999</v>
+      </c>
+      <c r="K39">
+        <v>20405.064514286099</v>
+      </c>
+      <c r="L39">
+        <v>25730.040652601801</v>
+      </c>
+      <c r="M39">
+        <v>34502.9768350472</v>
+      </c>
+      <c r="N39">
+        <v>1409.83742959549</v>
+      </c>
+      <c r="O39">
+        <v>0</v>
+      </c>
+      <c r="P39">
+        <v>0.71757732056978696</v>
+      </c>
+      <c r="Q39" s="3" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updating the files with 9000AF results
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
@@ -1,17 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\sweep results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9868276-1B3B-4482-8D6A-72B457499567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA57482E-4594-4EF8-92A5-118B128B7486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14503" yWindow="0" windowWidth="18497" windowHeight="17880" activeTab="2" xr2:uid="{526C491F-7D81-4CF8-8DF5-6D840C914C1B}"/>
-    <workbookView xWindow="-86" yWindow="0" windowWidth="14760" windowHeight="17880" activeTab="1" xr2:uid="{811D88E6-5E04-4AC4-9B26-930D2EA2E3F2}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{811D88E6-5E04-4AC4-9B26-930D2EA2E3F2}"/>
   </bookViews>
   <sheets>
     <sheet name="Summer Cost Summary" sheetId="4" r:id="rId1"/>
@@ -297,12 +296,17 @@
   <autoFilter ref="A1:Q39" xr:uid="{61A7BF30-9E2E-4F6C-9DD3-062B2A684BE6}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Winter"/>
+        <filter val="Summer"/>
       </filters>
     </filterColumn>
     <filterColumn colId="1">
       <filters>
         <filter val="0"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="3">
+      <filters>
+        <filter val="9000"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -730,7 +734,7 @@
         <v>211634.775495949</v>
       </c>
       <c r="D11" s="3">
-        <v>90145.456985227414</v>
+        <v>90280.635276184097</v>
       </c>
       <c r="F11" s="1"/>
     </row>
@@ -1231,7 +1235,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1239,7 +1243,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="3">
-        <f>N2+M2+L2+K2+J2</f>
+        <f t="shared" ref="C2:C39" si="0">N2+M2+L2+K2+J2</f>
         <v>158104.1957609462</v>
       </c>
       <c r="D2">
@@ -1293,7 +1297,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="3">
-        <f>N3+M3+L3+K3+J3</f>
+        <f t="shared" si="0"/>
         <v>171053.54809522501</v>
       </c>
       <c r="D3">
@@ -1347,7 +1351,7 @@
         <v>0</v>
       </c>
       <c r="C4" s="3">
-        <f>N4+M4+L4+K4+J4</f>
+        <f t="shared" si="0"/>
         <v>80541.55863</v>
       </c>
       <c r="D4">
@@ -1393,7 +1397,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1402,7 +1406,7 @@
       </c>
       <c r="C5" s="3">
         <f>N5+M5+L5+K5+J5</f>
-        <v>90145.456985227414</v>
+        <v>90280.635276184097</v>
       </c>
       <c r="D5">
         <v>9000</v>
@@ -1411,37 +1415,37 @@
         <v>10</v>
       </c>
       <c r="F5">
-        <v>211634.775495949</v>
+        <v>211634.75342465701</v>
       </c>
       <c r="G5">
-        <v>210256.540792755</v>
+        <v>210417.696825046</v>
       </c>
       <c r="H5">
-        <v>14871.657722592799</v>
+        <v>14646.6764757971</v>
       </c>
       <c r="I5">
-        <v>6315.0305970216004</v>
+        <v>8813.4656236474493</v>
       </c>
       <c r="J5">
-        <v>38197.462944573999</v>
+        <v>38471.8456521587</v>
       </c>
       <c r="K5">
-        <v>14447.7282003115</v>
+        <v>12390.141217574101</v>
       </c>
       <c r="L5">
-        <v>14872.6788013735</v>
+        <v>14543.585328987299</v>
       </c>
       <c r="M5">
-        <v>21186.688319614401</v>
+        <v>23460.1420994445</v>
       </c>
       <c r="N5">
-        <v>1440.8987193540199</v>
+        <v>1414.9209780195099</v>
       </c>
       <c r="O5">
-        <v>0.215568862275449</v>
+        <v>3.59281437125748E-2</v>
       </c>
       <c r="P5">
-        <v>0.99348767375321601</v>
+        <v>0.99424925925483998</v>
       </c>
       <c r="Q5" s="3" t="s">
         <v>25</v>
@@ -1455,7 +1459,7 @@
         <v>0</v>
       </c>
       <c r="C6" s="3">
-        <f>N6+M6+L6+K6+J6</f>
+        <f t="shared" si="0"/>
         <v>99135.784106883366</v>
       </c>
       <c r="D6">
@@ -1509,7 +1513,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="3">
-        <f>N7+M7+L7+K7+J7</f>
+        <f t="shared" si="0"/>
         <v>28772.571914996501</v>
       </c>
       <c r="D7">
@@ -1560,7 +1564,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="3">
-        <f>N8+M8+L8+K8+J8</f>
+        <f t="shared" si="0"/>
         <v>22368.52857086459</v>
       </c>
       <c r="D8">
@@ -1611,7 +1615,7 @@
         <v>5</v>
       </c>
       <c r="C9" s="3">
-        <f>N9+M9+L9+K9+J9</f>
+        <f t="shared" si="0"/>
         <v>16720.240035535448</v>
       </c>
       <c r="D9">
@@ -1662,7 +1666,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="3">
-        <f>N10+M10+L10+K10+J10</f>
+        <f t="shared" si="0"/>
         <v>108042.46335199999</v>
       </c>
       <c r="D10">
@@ -1716,7 +1720,7 @@
         <v>3</v>
       </c>
       <c r="C11" s="3">
-        <f>N11+M11+L11+K11+J11</f>
+        <f t="shared" si="0"/>
         <v>41752.231305558547</v>
       </c>
       <c r="D11">
@@ -1767,7 +1771,7 @@
         <v>3</v>
       </c>
       <c r="C12" s="3">
-        <f>N12+M12+L12+K12+J12</f>
+        <f t="shared" si="0"/>
         <v>51495.778789739757</v>
       </c>
       <c r="D12">
@@ -1818,7 +1822,7 @@
         <v>3</v>
       </c>
       <c r="C13" s="3">
-        <f>N13+M13+L13+K13+J13</f>
+        <f t="shared" si="0"/>
         <v>60724.979693855727</v>
       </c>
       <c r="D13">
@@ -1869,7 +1873,7 @@
         <v>3</v>
       </c>
       <c r="C14" s="3">
-        <f>N14+M14+L14+K14+J14</f>
+        <f t="shared" si="0"/>
         <v>70388.430895292957</v>
       </c>
       <c r="D14">
@@ -1920,7 +1924,7 @@
         <v>3</v>
       </c>
       <c r="C15" s="3">
-        <f>N15+M15+L15+K15+J15</f>
+        <f t="shared" si="0"/>
         <v>80116.314065181752</v>
       </c>
       <c r="D15">
@@ -1971,7 +1975,7 @@
         <v>3</v>
       </c>
       <c r="C16" s="3">
-        <f>N16+M16+L16+K16+J16</f>
+        <f t="shared" si="0"/>
         <v>90891.797768890829</v>
       </c>
       <c r="D16">
@@ -2022,7 +2026,7 @@
         <v>0</v>
       </c>
       <c r="C17" s="3">
-        <f>N17+M17+L17+K17+J17</f>
+        <f t="shared" si="0"/>
         <v>117856.65704778227</v>
       </c>
       <c r="D17">
@@ -2076,7 +2080,7 @@
         <v>0</v>
       </c>
       <c r="C18" s="3">
-        <f>N18+M18+L18+K18+J18</f>
+        <f t="shared" si="0"/>
         <v>126980.73146875472</v>
       </c>
       <c r="D18">
@@ -2130,7 +2134,7 @@
         <v>0</v>
       </c>
       <c r="C19" s="3">
-        <f>N19+M19+L19+K19+J19</f>
+        <f t="shared" si="0"/>
         <v>135947.17095224367</v>
       </c>
       <c r="D19">
@@ -2176,7 +2180,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2184,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="C20" s="3">
-        <f>N20+M20+L20+K20+J20</f>
+        <f t="shared" si="0"/>
         <v>75506.612155252791</v>
       </c>
       <c r="D20">
@@ -2230,7 +2234,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -2238,7 +2242,7 @@
         <v>0</v>
       </c>
       <c r="C21" s="3">
-        <f>N21+M21+L21+K21+J21</f>
+        <f t="shared" si="0"/>
         <v>85155.50909649636</v>
       </c>
       <c r="D21">
@@ -2292,7 +2296,7 @@
         <v>0</v>
       </c>
       <c r="C22" s="3">
-        <f>N22+M22+L22+K22+J22</f>
+        <f t="shared" si="0"/>
         <v>146231.12922675692</v>
       </c>
       <c r="D22">
@@ -2346,7 +2350,7 @@
         <v>0</v>
       </c>
       <c r="C23" s="3">
-        <f>N23+M23+L23+K23+J23</f>
+        <f t="shared" si="0"/>
         <v>159412.81974307698</v>
       </c>
       <c r="D23">
@@ -2392,7 +2396,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>19</v>
       </c>
@@ -2400,7 +2404,7 @@
         <v>0</v>
       </c>
       <c r="C24" s="3">
-        <f>N24+M24+L24+K24+J24</f>
+        <f t="shared" si="0"/>
         <v>93848.445066986911</v>
       </c>
       <c r="D24">
@@ -2454,7 +2458,7 @@
         <v>0</v>
       </c>
       <c r="C25" s="3">
-        <f>N25+M25+L25+K25+J25</f>
+        <f t="shared" si="0"/>
         <v>81475.122661244794</v>
       </c>
       <c r="D25">
@@ -2500,7 +2504,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -2508,7 +2512,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="3">
-        <f>N26+M26+L26+K26+J26</f>
+        <f t="shared" si="0"/>
         <v>120337.96252123939</v>
       </c>
       <c r="D26">
@@ -2562,7 +2566,7 @@
         <v>0</v>
       </c>
       <c r="C27" s="3">
-        <f>N27+M27+L27+K27+J27</f>
+        <f t="shared" si="0"/>
         <v>120337.96252123939</v>
       </c>
       <c r="D27">
@@ -2616,7 +2620,7 @@
         <v>0</v>
       </c>
       <c r="C28" s="3">
-        <f>N28+M28+L28+K28+J28</f>
+        <f t="shared" si="0"/>
         <v>120337.96252123939</v>
       </c>
       <c r="D28">
@@ -2670,7 +2674,7 @@
         <v>0</v>
       </c>
       <c r="C29" s="3">
-        <f>N29+M29+L29+K29+J29</f>
+        <f t="shared" si="0"/>
         <v>121509.10762980059</v>
       </c>
       <c r="D29">
@@ -2724,7 +2728,7 @@
         <v>0</v>
       </c>
       <c r="C30" s="3">
-        <f>N30+M30+L30+K30+J30</f>
+        <f t="shared" si="0"/>
         <v>160240.68755374721</v>
       </c>
       <c r="D30">
@@ -2778,7 +2782,7 @@
         <v>0</v>
       </c>
       <c r="C31" s="3">
-        <f>N31+M31+L31+K31+J31</f>
+        <f t="shared" si="0"/>
         <v>160240.68755374721</v>
       </c>
       <c r="D31">
@@ -2832,7 +2836,7 @@
         <v>0</v>
       </c>
       <c r="C32" s="3">
-        <f>N32+M32+L32+K32+J32</f>
+        <f t="shared" si="0"/>
         <v>160240.68755374721</v>
       </c>
       <c r="D32">
@@ -2886,7 +2890,7 @@
         <v>0</v>
       </c>
       <c r="C33" s="3">
-        <f>N33+M33+L33+K33+J33</f>
+        <f t="shared" si="0"/>
         <v>161854.2162878394</v>
       </c>
       <c r="D33">
@@ -2932,7 +2936,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>19</v>
       </c>
@@ -2940,7 +2944,7 @@
         <v>0</v>
       </c>
       <c r="C34" s="3">
-        <f>N34+M34+L34+K34+J34</f>
+        <f t="shared" si="0"/>
         <v>102961.15922754805</v>
       </c>
       <c r="D34">
@@ -2986,7 +2990,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>19</v>
       </c>
@@ -2994,7 +2998,7 @@
         <v>0</v>
       </c>
       <c r="C35" s="3">
-        <f>N35+M35+L35+K35+J35</f>
+        <f t="shared" si="0"/>
         <v>112554.99851567688</v>
       </c>
       <c r="D35">
@@ -3038,7 +3042,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>19</v>
       </c>
@@ -3046,7 +3050,7 @@
         <v>0</v>
       </c>
       <c r="C36" s="3">
-        <f>N36+M36+L36+K36+J36</f>
+        <f t="shared" si="0"/>
         <v>121344.56621300505</v>
       </c>
       <c r="D36">
@@ -3092,7 +3096,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>19</v>
       </c>
@@ -3100,7 +3104,7 @@
         <v>0</v>
       </c>
       <c r="C37" s="3">
-        <f>N37+M37+L37+K37+J37</f>
+        <f t="shared" si="0"/>
         <v>130424.39365381806</v>
       </c>
       <c r="D37">
@@ -3146,7 +3150,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>19</v>
       </c>
@@ -3154,7 +3158,7 @@
         <v>0</v>
       </c>
       <c r="C38" s="3">
-        <f>N38+M38+L38+K38+J38</f>
+        <f t="shared" si="0"/>
         <v>140645.20979357499</v>
       </c>
       <c r="D38">
@@ -3200,7 +3204,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>19</v>
       </c>
@@ -3208,7 +3212,7 @@
         <v>0</v>
       </c>
       <c r="C39" s="3">
-        <f>N39+M39+L39+K39+J39</f>
+        <f t="shared" si="0"/>
         <v>149838.83143944858</v>
       </c>
       <c r="D39">

</xml_diff>

<commit_message>
Updating the annual analysis script and plots
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
+++ b/tutorials/flex_ro/sweep results/water_targ_sweep_ALL_RESULTS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\sweep results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA57482E-4594-4EF8-92A5-118B128B7486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A48E7D25-833C-4631-BC61-2F4BFB338A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{811D88E6-5E04-4AC4-9B26-930D2EA2E3F2}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{811D88E6-5E04-4AC4-9B26-930D2EA2E3F2}"/>
   </bookViews>
   <sheets>
     <sheet name="Summer Cost Summary" sheetId="4" r:id="rId1"/>
@@ -624,24 +624,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B1DDFCB-CD48-4284-8222-18B5894FE623}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.453125" customWidth="1"/>
-    <col min="4" max="4" width="9.81640625" customWidth="1"/>
-    <col min="5" max="5" width="9.453125" customWidth="1"/>
-    <col min="6" max="6" width="10.36328125" customWidth="1"/>
+    <col min="2" max="2" width="9.23046875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.4609375" customWidth="1"/>
+    <col min="4" max="4" width="9.84375" customWidth="1"/>
+    <col min="5" max="5" width="9.4609375" customWidth="1"/>
+    <col min="6" max="6" width="10.3828125" customWidth="1"/>
     <col min="7" max="7" width="18" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.4">
       <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="6"/>
       <c r="F1" s="6"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.4">
       <c r="D2">
         <v>0</v>
       </c>
@@ -652,7 +652,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B3" t="s">
         <v>0</v>
       </c>
@@ -660,7 +660,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -674,7 +674,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B5" s="3">
         <f>C5/$G$10</f>
         <v>1798.4286079070769</v>
@@ -685,7 +685,7 @@
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B6" s="3">
         <f>C6/$G$10</f>
         <v>2397.9615120043568</v>
@@ -695,22 +695,22 @@
       </c>
       <c r="D6" s="1"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.4">
       <c r="D7" s="1"/>
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.4">
       <c r="D8" s="1"/>
       <c r="F8" s="1"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.4">
       <c r="D9" s="1"/>
       <c r="F9" s="1"/>
       <c r="G9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B10">
         <v>8000</v>
       </c>
@@ -726,7 +726,7 @@
         <v>23.514972912500003</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B11">
         <v>9000</v>
       </c>
@@ -738,7 +738,7 @@
       </c>
       <c r="F11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.4">
       <c r="B12" s="3">
         <f>C12/$G$10</f>
         <v>9591.8460480174272</v>
@@ -749,7 +749,7 @@
       <c r="D12" s="1"/>
       <c r="F12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B13">
         <v>10000</v>
       </c>
@@ -762,7 +762,7 @@
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B14">
         <v>11000</v>
       </c>
@@ -775,7 +775,7 @@
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B15">
         <v>12000</v>
       </c>
@@ -788,7 +788,7 @@
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.4">
       <c r="B16">
         <v>13000</v>
       </c>
@@ -801,7 +801,7 @@
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B17">
         <v>14000</v>
       </c>
@@ -814,7 +814,7 @@
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B18">
         <v>15000</v>
       </c>
@@ -827,7 +827,7 @@
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.4">
       <c r="B19">
         <v>16000</v>
       </c>
@@ -840,7 +840,7 @@
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>3</v>
       </c>
@@ -857,7 +857,7 @@
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.4">
       <c r="C21">
         <f>C20*4/7</f>
         <v>225552</v>
@@ -868,30 +868,31 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E02D5E1-F801-4839-8C05-CA5C31CB2DFA}">
   <dimension ref="B1:H22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="3" max="3" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.453125" customWidth="1"/>
-    <col min="5" max="5" width="9.81640625" customWidth="1"/>
-    <col min="6" max="6" width="9.453125" customWidth="1"/>
-    <col min="7" max="7" width="10.36328125" customWidth="1"/>
+    <col min="3" max="3" width="9.23046875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.4609375" customWidth="1"/>
+    <col min="5" max="5" width="9.84375" customWidth="1"/>
+    <col min="6" max="6" width="9.4609375" customWidth="1"/>
+    <col min="7" max="7" width="10.3828125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:8" x14ac:dyDescent="0.4">
       <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="6"/>
       <c r="G1" s="6"/>
     </row>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.4">
       <c r="E2">
         <v>0</v>
       </c>
@@ -902,7 +903,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C3" t="s">
         <v>0</v>
       </c>
@@ -910,7 +911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.4">
       <c r="B4" t="s">
         <v>4</v>
       </c>
@@ -926,7 +927,7 @@
         <v>16720.240035535448</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C5">
         <v>1798</v>
       </c>
@@ -939,7 +940,7 @@
         <v>22368.52857086459</v>
       </c>
     </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C6">
         <v>2398</v>
       </c>
@@ -952,7 +953,7 @@
         <v>28772.571914996501</v>
       </c>
     </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C7">
         <v>3000</v>
       </c>
@@ -961,7 +962,7 @@
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
     </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C8">
         <v>4000</v>
       </c>
@@ -974,7 +975,7 @@
       </c>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C9">
         <v>5000</v>
       </c>
@@ -987,7 +988,7 @@
       </c>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C10">
         <v>6000</v>
       </c>
@@ -1003,7 +1004,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C11">
         <v>7000</v>
       </c>
@@ -1016,7 +1017,7 @@
       </c>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C12">
         <v>8000</v>
       </c>
@@ -1035,7 +1036,7 @@
         <v>23.514972602724001</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C13">
         <v>9000</v>
       </c>
@@ -1050,7 +1051,7 @@
       </c>
       <c r="G13" s="1"/>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C14" s="3">
         <f>D14/H12</f>
         <v>9591.8461743762273</v>
@@ -1061,52 +1062,69 @@
       <c r="E14" s="1"/>
       <c r="G14" s="1"/>
     </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C15">
         <v>10000</v>
       </c>
+      <c r="D15" s="3">
+        <f>C15*$H$12</f>
+        <v>235149.72602724002</v>
+      </c>
       <c r="E15">
         <v>93848</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:8" x14ac:dyDescent="0.4">
       <c r="C16">
         <v>11000</v>
       </c>
+      <c r="D16" s="3">
+        <f t="shared" ref="D16:D22" si="0">C16*$H$12</f>
+        <v>258664.698629964</v>
+      </c>
       <c r="E16" s="3">
         <v>102961.15922754805</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.4">
       <c r="C17">
         <v>12000</v>
       </c>
+      <c r="D17" s="3">
+        <f t="shared" si="0"/>
+        <v>282179.67123268801</v>
+      </c>
       <c r="E17">
         <v>112554.99851567688</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.4">
       <c r="C18">
         <v>13000</v>
       </c>
+      <c r="D18" s="3">
+        <f t="shared" si="0"/>
+        <v>305694.64383541199</v>
+      </c>
       <c r="E18" s="3">
         <v>121344.56621300505</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.4">
       <c r="C19">
         <v>14000</v>
       </c>
       <c r="D19" s="3">
-        <v>329240.017626649</v>
+        <f t="shared" si="0"/>
+        <v>329209.61643813603</v>
       </c>
       <c r="E19" s="3">
         <v>130424.39365381806</v>
@@ -1114,35 +1132,44 @@
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.4">
       <c r="C20">
         <v>15000</v>
       </c>
+      <c r="D20" s="3">
+        <f t="shared" si="0"/>
+        <v>352724.58904086001</v>
+      </c>
       <c r="E20" s="3">
         <v>140645.20979357499</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.4">
       <c r="C21">
         <v>16000</v>
       </c>
+      <c r="D21" s="3">
+        <f t="shared" si="0"/>
+        <v>376239.56164358399</v>
+      </c>
       <c r="E21" s="3">
         <v>149838.83143944858</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.4">
       <c r="B22" t="s">
         <v>3</v>
       </c>
       <c r="C22" s="3">
         <v>16785.730584030498</v>
       </c>
-      <c r="D22">
-        <v>394716</v>
+      <c r="D22" s="3">
+        <f t="shared" si="0"/>
+        <v>394715.99480018351</v>
       </c>
       <c r="E22" s="3">
         <v>158104.1957609462</v>
@@ -1155,34 +1182,35 @@
     <mergeCell ref="E1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44889D92-5C1B-43B6-BE00-3D23C35CC93C}">
   <dimension ref="A1:Q39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="8.7265625" customWidth="1"/>
-    <col min="2" max="3" width="11.81640625" customWidth="1"/>
-    <col min="4" max="4" width="22.26953125" customWidth="1"/>
-    <col min="5" max="5" width="28.81640625" customWidth="1"/>
-    <col min="6" max="6" width="26.90625" customWidth="1"/>
+    <col min="1" max="1" width="8.69140625" customWidth="1"/>
+    <col min="2" max="3" width="11.84375" customWidth="1"/>
+    <col min="4" max="4" width="22.23046875" customWidth="1"/>
+    <col min="5" max="5" width="28.84375" customWidth="1"/>
+    <col min="6" max="6" width="26.921875" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
-    <col min="8" max="8" width="20.08984375" customWidth="1"/>
-    <col min="9" max="9" width="21.54296875" customWidth="1"/>
-    <col min="10" max="10" width="18.453125" customWidth="1"/>
-    <col min="11" max="11" width="18.81640625" customWidth="1"/>
+    <col min="8" max="8" width="20.07421875" customWidth="1"/>
+    <col min="9" max="9" width="21.53515625" customWidth="1"/>
+    <col min="10" max="10" width="18.4609375" customWidth="1"/>
+    <col min="11" max="11" width="18.84375" customWidth="1"/>
     <col min="12" max="12" width="22" customWidth="1"/>
-    <col min="13" max="13" width="22.54296875" customWidth="1"/>
-    <col min="14" max="14" width="25.36328125" customWidth="1"/>
-    <col min="15" max="15" width="19.1796875" customWidth="1"/>
-    <col min="16" max="16" width="28.6328125" customWidth="1"/>
-    <col min="17" max="17" width="16.26953125" style="3" customWidth="1"/>
+    <col min="13" max="13" width="22.53515625" customWidth="1"/>
+    <col min="14" max="14" width="25.3828125" customWidth="1"/>
+    <col min="15" max="15" width="19.15234375" customWidth="1"/>
+    <col min="16" max="16" width="28.61328125" customWidth="1"/>
+    <col min="17" max="17" width="16.23046875" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
@@ -1235,7 +1263,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1289,7 +1317,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -1343,7 +1371,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1397,7 +1425,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -1451,7 +1479,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1505,7 +1533,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -1556,7 +1584,7 @@
         <v>2.6406704469603199</v>
       </c>
     </row>
-    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1607,7 +1635,7 @@
         <v>3.36954571208561</v>
       </c>
     </row>
-    <row r="9" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1658,7 +1686,7 @@
         <v>4.8864727960722396</v>
       </c>
     </row>
-    <row r="10" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -1712,7 +1740,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>19</v>
       </c>
@@ -1763,7 +1791,7 @@
         <v>1.7211299327173799</v>
       </c>
     </row>
-    <row r="12" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -1814,7 +1842,7 @@
         <v>1.45968753918303</v>
       </c>
     </row>
-    <row r="13" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -1865,7 +1893,7 @@
         <v>1.2818199310829099</v>
       </c>
     </row>
-    <row r="14" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -1916,7 +1944,7 @@
         <v>1.15734642471583</v>
       </c>
     </row>
-    <row r="15" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>19</v>
       </c>
@@ -1967,7 +1995,7 @@
         <v>1.06438923423513</v>
       </c>
     </row>
-    <row r="16" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>19</v>
       </c>
@@ -2018,7 +2046,7 @@
         <v>0.99711288227329198</v>
       </c>
     </row>
-    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
         <v>21</v>
       </c>
@@ -2072,7 +2100,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -2126,7 +2154,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -2180,7 +2208,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2234,7 +2262,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -2288,7 +2316,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -2342,7 +2370,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -2396,7 +2424,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A24" t="s">
         <v>19</v>
       </c>
@@ -2450,7 +2478,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -2504,7 +2532,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.4">
       <c r="A26" t="s">
         <v>21</v>
       </c>
@@ -2558,7 +2586,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A27" t="s">
         <v>21</v>
       </c>
@@ -2612,7 +2640,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>21</v>
       </c>
@@ -2666,7 +2694,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>21</v>
       </c>
@@ -2720,7 +2748,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -2774,7 +2802,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -2828,7 +2856,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A32" t="s">
         <v>21</v>
       </c>
@@ -2882,7 +2910,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>21</v>
       </c>
@@ -2936,7 +2964,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>19</v>
       </c>
@@ -2990,7 +3018,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A35" t="s">
         <v>19</v>
       </c>
@@ -3042,7 +3070,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>19</v>
       </c>
@@ -3096,7 +3124,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>19</v>
       </c>
@@ -3150,7 +3178,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>19</v>
       </c>
@@ -3204,7 +3232,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" spans="1:17" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:17" hidden="1" x14ac:dyDescent="0.4">
       <c r="A39" t="s">
         <v>19</v>
       </c>

</xml_diff>